<commit_message>
starting to build out sdq queries
</commit_message>
<xml_diff>
--- a/spring-app/src/test/resources/Test File 1.xlsx
+++ b/spring-app/src/test/resources/Test File 1.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <fileSharing readOnlyRecommended="1"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586EC54B-7F13-2649-B42B-A43B901D68C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59B118D-5E99-2249-9DDF-F367552B2FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions for Use" sheetId="11" r:id="rId1"/>
@@ -1940,9 +1940,6 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1978,6 +1975,9 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -2022,22 +2022,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -2055,6 +2039,22 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -22433,19 +22433,19 @@
       <c r="D15" t="s">
         <v>173</v>
       </c>
-      <c r="F15" s="148" t="s">
+      <c r="F15" s="157" t="s">
         <v>157</v>
       </c>
-      <c r="G15" s="148"/>
-      <c r="H15" s="148"/>
-      <c r="I15" s="148"/>
-      <c r="J15" s="148"/>
-      <c r="K15" s="148"/>
-      <c r="L15" s="148"/>
-      <c r="M15" s="148"/>
-      <c r="N15" s="148"/>
-      <c r="O15" s="148"/>
-      <c r="P15" s="148"/>
+      <c r="G15" s="157"/>
+      <c r="H15" s="157"/>
+      <c r="I15" s="157"/>
+      <c r="J15" s="157"/>
+      <c r="K15" s="157"/>
+      <c r="L15" s="157"/>
+      <c r="M15" s="157"/>
+      <c r="N15" s="157"/>
+      <c r="O15" s="157"/>
+      <c r="P15" s="157"/>
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -29372,9 +29372,9 @@
       <c r="G9" s="133">
         <v>1</v>
       </c>
-      <c r="H9" s="50" t="str">
+      <c r="H9" s="50">
         <f>IF('SDQ Period 1'!D6="", "", 'SDQ Period 1'!D6)</f>
-        <v/>
+        <v>45885</v>
       </c>
     </row>
     <row r="10" spans="5:8" x14ac:dyDescent="0.2">
@@ -29385,9 +29385,9 @@
       <c r="G10" s="8">
         <v>2</v>
       </c>
-      <c r="H10" s="52" t="str">
+      <c r="H10" s="52">
         <f>IF('SDQ Period 2'!D6="", "", 'SDQ Period 2'!D6)</f>
-        <v/>
+        <v>45917</v>
       </c>
     </row>
     <row r="11" spans="5:8" x14ac:dyDescent="0.2">
@@ -29485,7 +29485,7 @@
     <row r="19" spans="5:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H19" s="85" t="str" cm="1">
         <f t="array" ref="H19">IF(COUNT(H9:H17)&lt;2, "", IF(SUMPRODUCT((ISNUMBER(H10:H17))*(ISNUMBER(H9:H16))*(H10:H17&lt;H9:H16))&gt;0, "⚠️ Not in Order", "✓ All in Order"))</f>
-        <v/>
+        <v>✓ All in Order</v>
       </c>
     </row>
   </sheetData>
@@ -33362,34 +33362,34 @@
       <c r="D7" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="F7" s="148" t="s">
+      <c r="F7" s="157" t="s">
         <v>157</v>
       </c>
-      <c r="G7" s="148"/>
-      <c r="H7" s="148"/>
-      <c r="I7" s="148"/>
-      <c r="J7" s="148"/>
-      <c r="K7" s="148"/>
-      <c r="L7" s="148"/>
-      <c r="M7" s="148"/>
-      <c r="N7" s="148"/>
-      <c r="O7" s="148"/>
-      <c r="P7" s="148"/>
+      <c r="G7" s="157"/>
+      <c r="H7" s="157"/>
+      <c r="I7" s="157"/>
+      <c r="J7" s="157"/>
+      <c r="K7" s="157"/>
+      <c r="L7" s="157"/>
+      <c r="M7" s="157"/>
+      <c r="N7" s="157"/>
+      <c r="O7" s="157"/>
+      <c r="P7" s="157"/>
       <c r="Q7" s="5"/>
     </row>
     <row r="8" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C8" s="4"/>
-      <c r="F8" s="148" t="s">
+      <c r="F8" s="157" t="s">
         <v>158</v>
       </c>
-      <c r="G8" s="148"/>
-      <c r="H8" s="148"/>
-      <c r="I8" s="148"/>
-      <c r="J8" s="148"/>
-      <c r="K8" s="148"/>
-      <c r="L8" s="148"/>
-      <c r="M8" s="148"/>
-      <c r="N8" s="148"/>
+      <c r="G8" s="157"/>
+      <c r="H8" s="157"/>
+      <c r="I8" s="157"/>
+      <c r="J8" s="157"/>
+      <c r="K8" s="157"/>
+      <c r="L8" s="157"/>
+      <c r="M8" s="157"/>
+      <c r="N8" s="157"/>
       <c r="O8" s="18"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="5"/>
@@ -33575,7 +33575,7 @@
       </c>
       <c r="E14" s="143" t="str">
         <f>IF('&lt;&lt;&lt;Summary SDQs by Period&gt;&gt;&gt;'!H19=0, "", '&lt;&lt;&lt;Summary SDQs by Period&gt;&gt;&gt;'!H19)</f>
-        <v/>
+        <v>✓ All in Order</v>
       </c>
       <c r="M14" s="24"/>
     </row>
@@ -33682,18 +33682,18 @@
     </row>
     <row r="26" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B26" s="23"/>
-      <c r="E26" s="152" t="s">
+      <c r="E26" s="151" t="s">
         <v>118</v>
       </c>
-      <c r="F26" s="154"/>
+      <c r="F26" s="153"/>
       <c r="G26" s="29"/>
-      <c r="H26" s="149" t="s">
+      <c r="H26" s="148" t="s">
         <v>119</v>
       </c>
-      <c r="I26" s="150"/>
-      <c r="J26" s="150"/>
-      <c r="K26" s="150"/>
-      <c r="L26" s="151"/>
+      <c r="I26" s="149"/>
+      <c r="J26" s="149"/>
+      <c r="K26" s="149"/>
+      <c r="L26" s="150"/>
       <c r="M26" s="24"/>
     </row>
     <row r="27" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -33705,13 +33705,13 @@
         <v>91</v>
       </c>
       <c r="G27" s="29"/>
-      <c r="H27" s="175" t="s">
+      <c r="H27" s="171" t="s">
         <v>123</v>
       </c>
-      <c r="I27" s="176"/>
-      <c r="J27" s="176"/>
-      <c r="K27" s="176"/>
-      <c r="L27" s="177"/>
+      <c r="I27" s="172"/>
+      <c r="J27" s="172"/>
+      <c r="K27" s="172"/>
+      <c r="L27" s="173"/>
       <c r="M27" s="24"/>
     </row>
     <row r="28" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -33751,9 +33751,9 @@
         <f>IF('Goal Based Outcomes (GBO)'!D13&lt;&gt;"", 'Goal Based Outcomes (GBO)'!D13, IF('Goal Based Outcomes (GBO)'!D36&lt;&gt;"", 'Goal Based Outcomes (GBO)'!D36, IF('Goal Based Outcomes (GBO)'!D59&lt;&gt;"", 'Goal Based Outcomes (GBO)'!D59, IF('Goal Based Outcomes (GBO)'!D82&lt;&gt;"",'Goal Based Outcomes (GBO)'!D82, ""))))</f>
         <v>45880</v>
       </c>
-      <c r="F29" s="50" t="str">
+      <c r="F29" s="50">
         <f>IF('SDQ Period 1'!D6&lt;&gt;"", 'SDQ Period 1'!D6, "")</f>
-        <v/>
+        <v>45885</v>
       </c>
       <c r="H29" s="37"/>
       <c r="I29" s="38"/>
@@ -33771,9 +33771,9 @@
         <f>IF('Goal Based Outcomes (GBO)'!D14&lt;&gt;"", 'Goal Based Outcomes (GBO)'!D14, IF('Goal Based Outcomes (GBO)'!D37&lt;&gt;"", 'Goal Based Outcomes (GBO)'!D37, IF('Goal Based Outcomes (GBO)'!D60&lt;&gt;"", 'Goal Based Outcomes (GBO)'!D60, IF('Goal Based Outcomes (GBO)'!D83&lt;&gt;"",'Goal Based Outcomes (GBO)'!D83, ""))))</f>
         <v/>
       </c>
-      <c r="F30" s="52" t="str">
+      <c r="F30" s="52">
         <f>IF('SDQ Period 2'!D6&lt;&gt;"", 'SDQ Period 2'!D6, "")</f>
-        <v/>
+        <v>45917</v>
       </c>
       <c r="H30" s="37"/>
       <c r="I30" s="38"/>
@@ -33969,15 +33969,15 @@
       <c r="E42" s="62" t="s">
         <v>142</v>
       </c>
-      <c r="F42" s="152" t="s">
+      <c r="F42" s="151" t="s">
         <v>154</v>
       </c>
-      <c r="G42" s="153"/>
-      <c r="H42" s="153"/>
-      <c r="I42" s="153"/>
-      <c r="J42" s="153"/>
-      <c r="K42" s="153"/>
-      <c r="L42" s="154"/>
+      <c r="G42" s="152"/>
+      <c r="H42" s="152"/>
+      <c r="I42" s="152"/>
+      <c r="J42" s="152"/>
+      <c r="K42" s="152"/>
+      <c r="L42" s="153"/>
       <c r="M42" s="24"/>
     </row>
     <row r="43" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -33998,13 +33998,13 @@
         <v>Complete</v>
       </c>
       <c r="E44" s="95"/>
-      <c r="F44" s="178"/>
-      <c r="G44" s="178"/>
-      <c r="H44" s="178"/>
-      <c r="I44" s="178"/>
-      <c r="J44" s="178"/>
-      <c r="K44" s="178"/>
-      <c r="L44" s="179"/>
+      <c r="F44" s="174"/>
+      <c r="G44" s="174"/>
+      <c r="H44" s="174"/>
+      <c r="I44" s="174"/>
+      <c r="J44" s="174"/>
+      <c r="K44" s="174"/>
+      <c r="L44" s="175"/>
       <c r="M44" s="24"/>
     </row>
     <row r="45" spans="2:13" ht="16" x14ac:dyDescent="0.2">
@@ -34019,13 +34019,13 @@
         <v>Incomplete</v>
       </c>
       <c r="E45" s="96"/>
-      <c r="F45" s="171"/>
-      <c r="G45" s="171"/>
-      <c r="H45" s="171"/>
-      <c r="I45" s="171"/>
-      <c r="J45" s="171"/>
-      <c r="K45" s="171"/>
-      <c r="L45" s="172"/>
+      <c r="F45" s="176"/>
+      <c r="G45" s="176"/>
+      <c r="H45" s="176"/>
+      <c r="I45" s="176"/>
+      <c r="J45" s="176"/>
+      <c r="K45" s="176"/>
+      <c r="L45" s="177"/>
       <c r="M45" s="24"/>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.2">
@@ -34038,13 +34038,13 @@
         <v>Incomplete</v>
       </c>
       <c r="E46" s="96"/>
-      <c r="F46" s="171"/>
-      <c r="G46" s="171"/>
-      <c r="H46" s="171"/>
-      <c r="I46" s="171"/>
-      <c r="J46" s="171"/>
-      <c r="K46" s="171"/>
-      <c r="L46" s="172"/>
+      <c r="F46" s="176"/>
+      <c r="G46" s="176"/>
+      <c r="H46" s="176"/>
+      <c r="I46" s="176"/>
+      <c r="J46" s="176"/>
+      <c r="K46" s="176"/>
+      <c r="L46" s="177"/>
       <c r="M46" s="24"/>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
@@ -34057,13 +34057,13 @@
         <v>Incomplete</v>
       </c>
       <c r="E47" s="96"/>
-      <c r="F47" s="171"/>
-      <c r="G47" s="171"/>
-      <c r="H47" s="171"/>
-      <c r="I47" s="171"/>
-      <c r="J47" s="171"/>
-      <c r="K47" s="171"/>
-      <c r="L47" s="172"/>
+      <c r="F47" s="176"/>
+      <c r="G47" s="176"/>
+      <c r="H47" s="176"/>
+      <c r="I47" s="176"/>
+      <c r="J47" s="176"/>
+      <c r="K47" s="176"/>
+      <c r="L47" s="177"/>
       <c r="M47" s="24"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.2">
@@ -34076,13 +34076,13 @@
         <v/>
       </c>
       <c r="E48" s="96"/>
-      <c r="F48" s="171"/>
-      <c r="G48" s="171"/>
-      <c r="H48" s="171"/>
-      <c r="I48" s="171"/>
-      <c r="J48" s="171"/>
-      <c r="K48" s="171"/>
-      <c r="L48" s="172"/>
+      <c r="F48" s="176"/>
+      <c r="G48" s="176"/>
+      <c r="H48" s="176"/>
+      <c r="I48" s="176"/>
+      <c r="J48" s="176"/>
+      <c r="K48" s="176"/>
+      <c r="L48" s="177"/>
       <c r="M48" s="24"/>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.2">
@@ -34095,13 +34095,13 @@
         <v/>
       </c>
       <c r="E49" s="96"/>
-      <c r="F49" s="171"/>
-      <c r="G49" s="171"/>
-      <c r="H49" s="171"/>
-      <c r="I49" s="171"/>
-      <c r="J49" s="171"/>
-      <c r="K49" s="171"/>
-      <c r="L49" s="172"/>
+      <c r="F49" s="176"/>
+      <c r="G49" s="176"/>
+      <c r="H49" s="176"/>
+      <c r="I49" s="176"/>
+      <c r="J49" s="176"/>
+      <c r="K49" s="176"/>
+      <c r="L49" s="177"/>
       <c r="M49" s="24"/>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.2">
@@ -34114,13 +34114,13 @@
         <v/>
       </c>
       <c r="E50" s="96"/>
-      <c r="F50" s="171"/>
-      <c r="G50" s="171"/>
-      <c r="H50" s="171"/>
-      <c r="I50" s="171"/>
-      <c r="J50" s="171"/>
-      <c r="K50" s="171"/>
-      <c r="L50" s="172"/>
+      <c r="F50" s="176"/>
+      <c r="G50" s="176"/>
+      <c r="H50" s="176"/>
+      <c r="I50" s="176"/>
+      <c r="J50" s="176"/>
+      <c r="K50" s="176"/>
+      <c r="L50" s="177"/>
       <c r="M50" s="24"/>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.2">
@@ -34133,13 +34133,13 @@
         <v/>
       </c>
       <c r="E51" s="96"/>
-      <c r="F51" s="171"/>
-      <c r="G51" s="171"/>
-      <c r="H51" s="171"/>
-      <c r="I51" s="171"/>
-      <c r="J51" s="171"/>
-      <c r="K51" s="171"/>
-      <c r="L51" s="172"/>
+      <c r="F51" s="176"/>
+      <c r="G51" s="176"/>
+      <c r="H51" s="176"/>
+      <c r="I51" s="176"/>
+      <c r="J51" s="176"/>
+      <c r="K51" s="176"/>
+      <c r="L51" s="177"/>
       <c r="M51" s="24"/>
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.2">
@@ -34152,13 +34152,13 @@
         <v/>
       </c>
       <c r="E52" s="96"/>
-      <c r="F52" s="171"/>
-      <c r="G52" s="171"/>
-      <c r="H52" s="171"/>
-      <c r="I52" s="171"/>
-      <c r="J52" s="171"/>
-      <c r="K52" s="171"/>
-      <c r="L52" s="172"/>
+      <c r="F52" s="176"/>
+      <c r="G52" s="176"/>
+      <c r="H52" s="176"/>
+      <c r="I52" s="176"/>
+      <c r="J52" s="176"/>
+      <c r="K52" s="176"/>
+      <c r="L52" s="177"/>
       <c r="M52" s="24"/>
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.2">
@@ -34171,13 +34171,13 @@
         <v/>
       </c>
       <c r="E53" s="96"/>
-      <c r="F53" s="171"/>
-      <c r="G53" s="171"/>
-      <c r="H53" s="171"/>
-      <c r="I53" s="171"/>
-      <c r="J53" s="171"/>
-      <c r="K53" s="171"/>
-      <c r="L53" s="172"/>
+      <c r="F53" s="176"/>
+      <c r="G53" s="176"/>
+      <c r="H53" s="176"/>
+      <c r="I53" s="176"/>
+      <c r="J53" s="176"/>
+      <c r="K53" s="176"/>
+      <c r="L53" s="177"/>
       <c r="M53" s="24"/>
     </row>
     <row r="54" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -34190,13 +34190,13 @@
         <v/>
       </c>
       <c r="E54" s="97"/>
-      <c r="F54" s="173"/>
-      <c r="G54" s="173"/>
-      <c r="H54" s="173"/>
-      <c r="I54" s="173"/>
-      <c r="J54" s="173"/>
-      <c r="K54" s="173"/>
-      <c r="L54" s="174"/>
+      <c r="F54" s="178"/>
+      <c r="G54" s="178"/>
+      <c r="H54" s="178"/>
+      <c r="I54" s="178"/>
+      <c r="J54" s="178"/>
+      <c r="K54" s="178"/>
+      <c r="L54" s="179"/>
       <c r="M54" s="24"/>
     </row>
     <row r="55" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -34231,21 +34231,21 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="meQlOIUyLBIuMEmLULxOJ5BN6ywfQKo/ce77jYeQOok4oymmYE6uhv4CE50s1CJqAdhs10ldO7sl02oDeL3B4Q==" saltValue="S188sJ2TnHkDHo5hfVrlJg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="15">
+    <mergeCell ref="F50:L50"/>
+    <mergeCell ref="F51:L51"/>
+    <mergeCell ref="F52:L52"/>
+    <mergeCell ref="F53:L53"/>
+    <mergeCell ref="F54:L54"/>
+    <mergeCell ref="F45:L45"/>
+    <mergeCell ref="F46:L46"/>
+    <mergeCell ref="F47:L47"/>
+    <mergeCell ref="F48:L48"/>
+    <mergeCell ref="F49:L49"/>
     <mergeCell ref="H26:L26"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="H27:L27"/>
     <mergeCell ref="F42:L42"/>
     <mergeCell ref="F44:L44"/>
-    <mergeCell ref="F45:L45"/>
-    <mergeCell ref="F46:L46"/>
-    <mergeCell ref="F47:L47"/>
-    <mergeCell ref="F48:L48"/>
-    <mergeCell ref="F49:L49"/>
-    <mergeCell ref="F50:L50"/>
-    <mergeCell ref="F51:L51"/>
-    <mergeCell ref="F52:L52"/>
-    <mergeCell ref="F53:L53"/>
-    <mergeCell ref="F54:L54"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="E21">
@@ -35130,14 +35130,14 @@
         <v>135</v>
       </c>
       <c r="D9" s="124"/>
-      <c r="E9" s="153" t="s">
+      <c r="E9" s="152" t="s">
         <v>134</v>
       </c>
-      <c r="F9" s="153"/>
-      <c r="G9" s="153"/>
-      <c r="H9" s="153"/>
-      <c r="I9" s="153"/>
-      <c r="J9" s="154"/>
+      <c r="F9" s="152"/>
+      <c r="G9" s="152"/>
+      <c r="H9" s="152"/>
+      <c r="I9" s="152"/>
+      <c r="J9" s="153"/>
     </row>
     <row r="10" spans="3:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E10" s="60">
@@ -35166,14 +35166,14 @@
       <c r="H11" s="63"/>
       <c r="I11" s="63"/>
       <c r="J11" s="63"/>
-      <c r="L11" s="149" t="s">
+      <c r="L11" s="148" t="s">
         <v>192</v>
       </c>
-      <c r="M11" s="150"/>
-      <c r="N11" s="150"/>
-      <c r="O11" s="150"/>
-      <c r="P11" s="150"/>
-      <c r="Q11" s="151"/>
+      <c r="M11" s="149"/>
+      <c r="N11" s="149"/>
+      <c r="O11" s="149"/>
+      <c r="P11" s="149"/>
+      <c r="Q11" s="150"/>
     </row>
     <row r="12" spans="3:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C12" s="113" t="s">
@@ -35887,14 +35887,14 @@
         <v>135</v>
       </c>
       <c r="D32" s="124"/>
-      <c r="E32" s="152" t="s">
+      <c r="E32" s="151" t="s">
         <v>137</v>
       </c>
-      <c r="F32" s="153"/>
-      <c r="G32" s="153"/>
-      <c r="H32" s="153"/>
-      <c r="I32" s="153"/>
-      <c r="J32" s="154"/>
+      <c r="F32" s="152"/>
+      <c r="G32" s="152"/>
+      <c r="H32" s="152"/>
+      <c r="I32" s="152"/>
+      <c r="J32" s="153"/>
       <c r="L32"/>
       <c r="M32"/>
       <c r="N32"/>
@@ -35989,12 +35989,12 @@
       <c r="J35" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="L35" s="155" t="s">
+      <c r="L35" s="154" t="s">
         <v>193</v>
       </c>
-      <c r="M35" s="156"/>
-      <c r="N35" s="156"/>
-      <c r="O35" s="157"/>
+      <c r="M35" s="155"/>
+      <c r="N35" s="155"/>
+      <c r="O35" s="156"/>
       <c r="P35" s="25"/>
       <c r="Q35" s="138" t="s">
         <v>196</v>
@@ -36506,14 +36506,14 @@
     </row>
     <row r="54" spans="2:15" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="2:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E55" s="152" t="s">
+      <c r="E55" s="151" t="s">
         <v>120</v>
       </c>
-      <c r="F55" s="153"/>
-      <c r="G55" s="153"/>
-      <c r="H55" s="153"/>
-      <c r="I55" s="153"/>
-      <c r="J55" s="154"/>
+      <c r="F55" s="152"/>
+      <c r="G55" s="152"/>
+      <c r="H55" s="152"/>
+      <c r="I55" s="152"/>
+      <c r="J55" s="153"/>
     </row>
     <row r="56" spans="2:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E56" s="60">
@@ -36788,14 +36788,14 @@
     </row>
     <row r="77" spans="3:10" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="78" spans="3:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E78" s="152" t="s">
+      <c r="E78" s="151" t="s">
         <v>133</v>
       </c>
-      <c r="F78" s="153"/>
-      <c r="G78" s="153"/>
-      <c r="H78" s="153"/>
-      <c r="I78" s="153"/>
-      <c r="J78" s="154"/>
+      <c r="F78" s="152"/>
+      <c r="G78" s="152"/>
+      <c r="H78" s="152"/>
+      <c r="I78" s="152"/>
+      <c r="J78" s="153"/>
     </row>
     <row r="79" spans="3:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E79" s="60">
@@ -37168,7 +37168,9 @@
       <c r="C6" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="D6" s="28"/>
+      <c r="D6" s="28">
+        <v>45885</v>
+      </c>
       <c r="E6" s="27"/>
     </row>
     <row r="7" spans="2:18" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -39077,7 +39079,9 @@
       <c r="C6" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="D6" s="28"/>
+      <c r="D6" s="28">
+        <v>45917</v>
+      </c>
     </row>
     <row r="7" spans="2:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="F7" s="26"/>

</xml_diff>